<commit_message>
Tower film: the hoist beat moves the hook, not the rope
Lengthening the drop from 26 m to 36 m changed nothing you could see -
the rope got longer and the hook stayed a speck near the ground. Shortened
to 5 m instead, the hook climbs to just under the jib and the ground
clearance goes 12.1 -> 33.1 m, which reads at a glance.

A second move follows in the same row: Trolley R 30 -> 10 m runs the
trolley and its hook back in along the jib toward the mast. Both cells sit
side by side under HOIST, so one card carries both.

Checked from a fixed camera before committing to it - which is the only
way to tell, since the engine re-fits on every load and would have hidden
the difference either way.
</commit_message>
<xml_diff>
--- a/plate3d/video/TOWER_3_HOOK.xlsx
+++ b/plate3d/video/TOWER_3_HOOK.xlsx
@@ -2061,7 +2061,7 @@
         <v>30000</v>
       </c>
       <c r="D19" s="8">
-        <v>36000</v>
+        <v>5000</v>
       </c>
       <c r="H19" s="9">
         <f>=PARAM!$J$12+1880</f>
@@ -2069,11 +2069,11 @@
       </c>
       <c r="I19" s="9">
         <f>=PARAM!$H$19-PARAM!$D$19</f>
-        <v>4020</v>
+        <v>35020</v>
       </c>
       <c r="J19" s="9">
         <f>=PARAM!$I$19-1910</f>
-        <v>2110</v>
+        <v>33110</v>
       </c>
     </row>
     <row r="20" spans="2:10" x14ac:dyDescent="0.25">
@@ -13122,7 +13122,7 @@
       </c>
       <c r="K305" s="18">
         <f>=PARAM!$D$19</f>
-        <v>36000</v>
+        <v>5000</v>
       </c>
       <c r="L305">
         <v>300</v>
@@ -13167,7 +13167,7 @@
       </c>
       <c r="K306" s="18">
         <f>=PARAM!$D$19</f>
-        <v>36000</v>
+        <v>5000</v>
       </c>
       <c r="L306">
         <v>300</v>
@@ -13212,7 +13212,7 @@
       </c>
       <c r="K307" s="18">
         <f>=PARAM!$D$19</f>
-        <v>36000</v>
+        <v>5000</v>
       </c>
       <c r="L307">
         <v>300</v>
@@ -13257,7 +13257,7 @@
       </c>
       <c r="K308" s="18">
         <f>=PARAM!$D$19</f>
-        <v>36000</v>
+        <v>5000</v>
       </c>
       <c r="L308">
         <v>300</v>
@@ -14381,7 +14381,7 @@
       </c>
       <c r="H346" s="18">
         <f>=PARAM!$I$19</f>
-        <v>4020</v>
+        <v>35020</v>
       </c>
       <c r="I346">
         <v>0</v>

</xml_diff>